<commit_message>
Add Quick Import for Excel; enhance RFQ generation & UI
Major update:
- Added RFQImportService for direct Excel pricesheet import (no Excel required)
- Implemented drag-and-drop UI for quick item import
- Improved Excel/PDF generation: template suffixes, page breaks, borders, currency handling
- Enhanced UI layout, dialogs, and error messages for clarity
- Updated quote code format for PO templates
- Added new NuGet packages and updated project references
- Improved folder selection and network fallback logic
- Refactored code for maintainability and future extensibility
</commit_message>
<xml_diff>
--- a/RFQ Generator Beta Version/Templates/DE TEMPLATE.xlsx
+++ b/RFQ Generator Beta Version/Templates/DE TEMPLATE.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\source\repos\RFQ Generator Beta Version\RFQ Generator Beta Version\bin\Debug\Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\source\repos\RFQ Generator Beta Version\RFQ Generator Beta Version\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1530A2F-8E46-4C75-BE15-81A29237B701}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EF364E6-594C-43C3-812F-068C5F37803E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{02CCD737-9343-44DD-A110-541534088332}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="51">
   <si>
     <t>ITEM</t>
   </si>
@@ -94,9 +94,6 @@
   </si>
   <si>
     <t xml:space="preserve">QTY </t>
-  </si>
-  <si>
-    <t>TOTAL RFQ VALUE</t>
   </si>
   <si>
     <t>DELIVERY</t>
@@ -303,7 +300,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -453,13 +450,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thick">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="100">
+  <cellXfs count="102">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -528,181 +536,197 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="39" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="39" fontId="5" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="4" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2127,92 +2151,92 @@
       <c r="T2" s="6"/>
     </row>
     <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="51"/>
-      <c r="B3" s="51"/>
-      <c r="C3" s="51"/>
-      <c r="D3" s="51"/>
-      <c r="E3" s="51"/>
-      <c r="F3" s="51"/>
-      <c r="G3" s="51"/>
-      <c r="H3" s="51"/>
-      <c r="I3" s="51"/>
-      <c r="J3" s="51"/>
-      <c r="K3" s="51"/>
-      <c r="L3" s="51"/>
-      <c r="M3" s="51"/>
-      <c r="N3" s="51"/>
-      <c r="O3" s="51"/>
-      <c r="P3" s="51"/>
-      <c r="Q3" s="51"/>
-      <c r="R3" s="51"/>
-      <c r="S3" s="51"/>
-      <c r="T3" s="51"/>
+      <c r="A3" s="55"/>
+      <c r="B3" s="55"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="55"/>
+      <c r="H3" s="55"/>
+      <c r="I3" s="55"/>
+      <c r="J3" s="55"/>
+      <c r="K3" s="55"/>
+      <c r="L3" s="55"/>
+      <c r="M3" s="55"/>
+      <c r="N3" s="55"/>
+      <c r="O3" s="55"/>
+      <c r="P3" s="55"/>
+      <c r="Q3" s="55"/>
+      <c r="R3" s="55"/>
+      <c r="S3" s="55"/>
+      <c r="T3" s="55"/>
     </row>
     <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="83"/>
-      <c r="B4" s="83"/>
-      <c r="C4" s="83"/>
-      <c r="D4" s="83"/>
-      <c r="E4" s="83"/>
-      <c r="F4" s="83"/>
-      <c r="G4" s="83"/>
-      <c r="H4" s="83"/>
-      <c r="I4" s="83"/>
-      <c r="J4" s="83"/>
-      <c r="K4" s="83"/>
-      <c r="L4" s="83"/>
-      <c r="M4" s="83"/>
-      <c r="N4" s="83"/>
-      <c r="O4" s="83"/>
-      <c r="P4" s="83"/>
-      <c r="Q4" s="83"/>
-      <c r="R4" s="83"/>
-      <c r="S4" s="83"/>
-      <c r="T4" s="83"/>
+      <c r="A4" s="56"/>
+      <c r="B4" s="56"/>
+      <c r="C4" s="56"/>
+      <c r="D4" s="56"/>
+      <c r="E4" s="56"/>
+      <c r="F4" s="56"/>
+      <c r="G4" s="56"/>
+      <c r="H4" s="56"/>
+      <c r="I4" s="56"/>
+      <c r="J4" s="56"/>
+      <c r="K4" s="56"/>
+      <c r="L4" s="56"/>
+      <c r="M4" s="56"/>
+      <c r="N4" s="56"/>
+      <c r="O4" s="56"/>
+      <c r="P4" s="56"/>
+      <c r="Q4" s="56"/>
+      <c r="R4" s="56"/>
+      <c r="S4" s="56"/>
+      <c r="T4" s="56"/>
     </row>
     <row r="5" spans="1:20" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="84"/>
-      <c r="B5" s="84"/>
-      <c r="C5" s="84"/>
-      <c r="D5" s="84"/>
-      <c r="E5" s="84"/>
-      <c r="F5" s="84"/>
-      <c r="G5" s="84"/>
-      <c r="H5" s="84"/>
-      <c r="I5" s="84"/>
-      <c r="J5" s="84"/>
-      <c r="K5" s="84"/>
-      <c r="L5" s="84"/>
-      <c r="M5" s="84"/>
-      <c r="N5" s="84"/>
-      <c r="O5" s="84"/>
-      <c r="P5" s="84"/>
-      <c r="Q5" s="84"/>
-      <c r="R5" s="84"/>
-      <c r="S5" s="84"/>
-      <c r="T5" s="84"/>
+      <c r="A5" s="57"/>
+      <c r="B5" s="57"/>
+      <c r="C5" s="57"/>
+      <c r="D5" s="57"/>
+      <c r="E5" s="57"/>
+      <c r="F5" s="57"/>
+      <c r="G5" s="57"/>
+      <c r="H5" s="57"/>
+      <c r="I5" s="57"/>
+      <c r="J5" s="57"/>
+      <c r="K5" s="57"/>
+      <c r="L5" s="57"/>
+      <c r="M5" s="57"/>
+      <c r="N5" s="57"/>
+      <c r="O5" s="57"/>
+      <c r="P5" s="57"/>
+      <c r="Q5" s="57"/>
+      <c r="R5" s="57"/>
+      <c r="S5" s="57"/>
+      <c r="T5" s="57"/>
     </row>
     <row r="6" spans="1:20" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="51"/>
-      <c r="B6" s="51"/>
-      <c r="C6" s="51"/>
-      <c r="D6" s="51"/>
-      <c r="E6" s="51"/>
-      <c r="F6" s="51"/>
-      <c r="G6" s="51"/>
-      <c r="H6" s="51"/>
-      <c r="I6" s="51"/>
-      <c r="J6" s="51"/>
-      <c r="K6" s="51"/>
-      <c r="L6" s="51"/>
-      <c r="M6" s="51"/>
-      <c r="N6" s="51"/>
-      <c r="O6" s="51"/>
-      <c r="P6" s="51"/>
-      <c r="Q6" s="51"/>
-      <c r="R6" s="51"/>
-      <c r="S6" s="51"/>
-      <c r="T6" s="51"/>
+      <c r="A6" s="55"/>
+      <c r="B6" s="55"/>
+      <c r="C6" s="55"/>
+      <c r="D6" s="55"/>
+      <c r="E6" s="55"/>
+      <c r="F6" s="55"/>
+      <c r="G6" s="55"/>
+      <c r="H6" s="55"/>
+      <c r="I6" s="55"/>
+      <c r="J6" s="55"/>
+      <c r="K6" s="55"/>
+      <c r="L6" s="55"/>
+      <c r="M6" s="55"/>
+      <c r="N6" s="55"/>
+      <c r="O6" s="55"/>
+      <c r="P6" s="55"/>
+      <c r="Q6" s="55"/>
+      <c r="R6" s="55"/>
+      <c r="S6" s="55"/>
+      <c r="T6" s="55"/>
     </row>
     <row r="7" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="7"/>
@@ -2311,7 +2335,7 @@
         <v>8</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H11" s="11" t="s">
         <v>9</v>
@@ -2325,7 +2349,7 @@
         <v>8</v>
       </c>
       <c r="N11" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="S11" s="10"/>
       <c r="T11" s="15"/>
@@ -2350,14 +2374,14 @@
       <c r="M12" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="N12" s="85" t="s">
-        <v>41</v>
-      </c>
-      <c r="O12" s="85"/>
-      <c r="P12" s="85"/>
-      <c r="Q12" s="85"/>
-      <c r="R12" s="85"/>
-      <c r="S12" s="85"/>
+      <c r="N12" s="58" t="s">
+        <v>40</v>
+      </c>
+      <c r="O12" s="58"/>
+      <c r="P12" s="58"/>
+      <c r="Q12" s="58"/>
+      <c r="R12" s="58"/>
+      <c r="S12" s="58"/>
       <c r="T12" s="17"/>
     </row>
     <row r="13" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -2379,7 +2403,7 @@
         <v>8</v>
       </c>
       <c r="N13" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T13" s="17"/>
     </row>
@@ -2391,10 +2415,10 @@
         <v>8</v>
       </c>
       <c r="E14" s="1"/>
-      <c r="K14" s="53"/>
-      <c r="L14" s="54"/>
-      <c r="M14" s="54"/>
-      <c r="N14" s="54"/>
+      <c r="K14" s="66"/>
+      <c r="L14" s="67"/>
+      <c r="M14" s="67"/>
+      <c r="N14" s="67"/>
       <c r="O14" s="1"/>
       <c r="P14" s="19"/>
       <c r="Q14" s="1"/>
@@ -2421,18 +2445,18 @@
       <c r="K15" s="8"/>
       <c r="L15" s="23"/>
       <c r="M15" s="8"/>
-      <c r="N15" s="69" t="s">
-        <v>25</v>
-      </c>
-      <c r="O15" s="69"/>
-      <c r="P15" s="69"/>
-      <c r="Q15" s="69"/>
-      <c r="R15" s="69"/>
-      <c r="S15" s="69"/>
-      <c r="T15" s="70"/>
+      <c r="N15" s="82" t="s">
+        <v>24</v>
+      </c>
+      <c r="O15" s="82"/>
+      <c r="P15" s="82"/>
+      <c r="Q15" s="82"/>
+      <c r="R15" s="82"/>
+      <c r="S15" s="82"/>
+      <c r="T15" s="83"/>
     </row>
     <row r="16" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="41"/>
+      <c r="A16" s="39"/>
       <c r="C16" s="1"/>
       <c r="E16" s="24"/>
       <c r="F16" s="24"/>
@@ -2447,238 +2471,238 @@
       <c r="T16" s="7"/>
     </row>
     <row r="17" spans="1:20" s="25" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="65" t="s">
+      <c r="A17" s="78" t="s">
         <v>0</v>
       </c>
-      <c r="B17" s="58"/>
-      <c r="C17" s="58" t="s">
+      <c r="B17" s="71"/>
+      <c r="C17" s="71" t="s">
         <v>18</v>
       </c>
-      <c r="D17" s="58"/>
-      <c r="E17" s="60" t="s">
+      <c r="D17" s="71"/>
+      <c r="E17" s="73" t="s">
         <v>1</v>
       </c>
-      <c r="F17" s="61"/>
-      <c r="G17" s="62"/>
-      <c r="H17" s="65" t="s">
-        <v>20</v>
-      </c>
-      <c r="I17" s="71"/>
-      <c r="J17" s="71"/>
-      <c r="K17" s="71"/>
-      <c r="L17" s="72"/>
-      <c r="M17" s="65" t="s">
+      <c r="F17" s="74"/>
+      <c r="G17" s="75"/>
+      <c r="H17" s="78" t="s">
+        <v>19</v>
+      </c>
+      <c r="I17" s="84"/>
+      <c r="J17" s="84"/>
+      <c r="K17" s="84"/>
+      <c r="L17" s="85"/>
+      <c r="M17" s="78" t="s">
         <v>2</v>
       </c>
-      <c r="N17" s="58"/>
-      <c r="O17" s="58"/>
-      <c r="P17" s="66"/>
-      <c r="Q17" s="65" t="s">
+      <c r="N17" s="71"/>
+      <c r="O17" s="71"/>
+      <c r="P17" s="79"/>
+      <c r="Q17" s="78" t="s">
         <v>11</v>
       </c>
-      <c r="R17" s="58"/>
-      <c r="S17" s="58"/>
-      <c r="T17" s="66"/>
+      <c r="R17" s="71"/>
+      <c r="S17" s="71"/>
+      <c r="T17" s="79"/>
     </row>
     <row r="18" spans="1:20" s="25" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="67"/>
-      <c r="B18" s="59"/>
-      <c r="C18" s="59"/>
-      <c r="D18" s="59"/>
-      <c r="E18" s="63"/>
-      <c r="F18" s="63"/>
-      <c r="G18" s="64"/>
-      <c r="H18" s="73"/>
-      <c r="I18" s="74"/>
-      <c r="J18" s="74"/>
-      <c r="K18" s="74"/>
-      <c r="L18" s="75"/>
-      <c r="M18" s="67"/>
-      <c r="N18" s="59"/>
-      <c r="O18" s="59"/>
-      <c r="P18" s="68"/>
-      <c r="Q18" s="67"/>
-      <c r="R18" s="59"/>
-      <c r="S18" s="59"/>
-      <c r="T18" s="68"/>
+      <c r="A18" s="80"/>
+      <c r="B18" s="72"/>
+      <c r="C18" s="72"/>
+      <c r="D18" s="72"/>
+      <c r="E18" s="76"/>
+      <c r="F18" s="76"/>
+      <c r="G18" s="77"/>
+      <c r="H18" s="86"/>
+      <c r="I18" s="87"/>
+      <c r="J18" s="87"/>
+      <c r="K18" s="87"/>
+      <c r="L18" s="88"/>
+      <c r="M18" s="80"/>
+      <c r="N18" s="72"/>
+      <c r="O18" s="72"/>
+      <c r="P18" s="81"/>
+      <c r="Q18" s="80"/>
+      <c r="R18" s="72"/>
+      <c r="S18" s="72"/>
+      <c r="T18" s="81"/>
     </row>
     <row r="19" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="81"/>
-      <c r="B19" s="82"/>
-      <c r="C19" s="81"/>
-      <c r="D19" s="82"/>
-      <c r="E19" s="86"/>
-      <c r="F19" s="87"/>
-      <c r="G19" s="88"/>
-      <c r="H19" s="81"/>
-      <c r="I19" s="93"/>
-      <c r="J19" s="93"/>
-      <c r="K19" s="93"/>
-      <c r="L19" s="82"/>
-      <c r="M19" s="81"/>
-      <c r="N19" s="93"/>
-      <c r="O19" s="93"/>
-      <c r="P19" s="82"/>
-      <c r="Q19" s="81"/>
-      <c r="R19" s="93"/>
-      <c r="S19" s="93"/>
-      <c r="T19" s="82"/>
+      <c r="A19" s="46"/>
+      <c r="B19" s="48"/>
+      <c r="C19" s="46"/>
+      <c r="D19" s="48"/>
+      <c r="E19" s="59"/>
+      <c r="F19" s="60"/>
+      <c r="G19" s="61"/>
+      <c r="H19" s="46"/>
+      <c r="I19" s="47"/>
+      <c r="J19" s="47"/>
+      <c r="K19" s="47"/>
+      <c r="L19" s="48"/>
+      <c r="M19" s="46"/>
+      <c r="N19" s="47"/>
+      <c r="O19" s="47"/>
+      <c r="P19" s="48"/>
+      <c r="Q19" s="46"/>
+      <c r="R19" s="47"/>
+      <c r="S19" s="47"/>
+      <c r="T19" s="48"/>
     </row>
     <row r="20" spans="1:20" s="18" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="76" t="s">
+      <c r="A20" s="62" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20" s="63"/>
+      <c r="C20" s="62" t="s">
         <v>43</v>
       </c>
-      <c r="B20" s="52"/>
-      <c r="C20" s="76" t="s">
+      <c r="D20" s="63"/>
+      <c r="E20" s="89" t="s">
         <v>44</v>
       </c>
-      <c r="D20" s="52"/>
-      <c r="E20" s="77" t="s">
+      <c r="F20" s="68"/>
+      <c r="G20" s="90"/>
+      <c r="H20" s="49" t="s">
         <v>45</v>
       </c>
-      <c r="F20" s="55"/>
-      <c r="G20" s="78"/>
-      <c r="H20" s="89" t="s">
+      <c r="I20" s="50"/>
+      <c r="J20" s="50"/>
+      <c r="K20" s="50"/>
+      <c r="L20" s="51"/>
+      <c r="M20" s="52" t="s">
         <v>46</v>
       </c>
-      <c r="I20" s="90"/>
-      <c r="J20" s="90"/>
-      <c r="K20" s="90"/>
-      <c r="L20" s="91"/>
-      <c r="M20" s="94" t="s">
+      <c r="N20" s="53"/>
+      <c r="O20" s="53"/>
+      <c r="P20" s="54"/>
+      <c r="Q20" s="52" t="s">
+        <v>33</v>
+      </c>
+      <c r="R20" s="53"/>
+      <c r="S20" s="53"/>
+      <c r="T20" s="54"/>
+    </row>
+    <row r="21" spans="1:20" s="18" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="43"/>
+      <c r="B21" s="45"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="45"/>
+      <c r="E21" s="40"/>
+      <c r="F21" s="41"/>
+      <c r="G21" s="42"/>
+      <c r="H21" s="43"/>
+      <c r="I21" s="44"/>
+      <c r="J21" s="44"/>
+      <c r="K21" s="44"/>
+      <c r="L21" s="45"/>
+      <c r="M21" s="43"/>
+      <c r="N21" s="44"/>
+      <c r="O21" s="44"/>
+      <c r="P21" s="45"/>
+      <c r="Q21" s="43"/>
+      <c r="R21" s="44"/>
+      <c r="S21" s="44"/>
+      <c r="T21" s="45"/>
+    </row>
+    <row r="22" spans="1:20" s="18" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="93"/>
+      <c r="B22" s="64"/>
+      <c r="C22" s="64"/>
+      <c r="D22" s="64"/>
+      <c r="E22" s="92"/>
+      <c r="F22" s="92"/>
+      <c r="G22" s="92"/>
+      <c r="H22" s="64" t="s">
+        <v>34</v>
+      </c>
+      <c r="I22" s="64"/>
+      <c r="J22" s="64"/>
+      <c r="K22" s="64"/>
+      <c r="L22" s="64"/>
+      <c r="M22" s="64"/>
+      <c r="N22" s="64"/>
+      <c r="O22" s="64"/>
+      <c r="P22" s="64"/>
+      <c r="Q22" s="64" t="s">
+        <v>36</v>
+      </c>
+      <c r="R22" s="64"/>
+      <c r="S22" s="64"/>
+      <c r="T22" s="65"/>
+    </row>
+    <row r="23" spans="1:20" s="18" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="97"/>
+      <c r="B23" s="98"/>
+      <c r="C23" s="55"/>
+      <c r="D23" s="55"/>
+      <c r="E23" s="91"/>
+      <c r="F23" s="91"/>
+      <c r="G23" s="91"/>
+      <c r="H23" s="55" t="s">
+        <v>35</v>
+      </c>
+      <c r="I23" s="55"/>
+      <c r="J23" s="55"/>
+      <c r="K23" s="55"/>
+      <c r="L23" s="55"/>
+      <c r="M23" s="55"/>
+      <c r="N23" s="55"/>
+      <c r="O23" s="55"/>
+      <c r="P23" s="55"/>
+      <c r="Q23" s="55" t="s">
+        <v>37</v>
+      </c>
+      <c r="R23" s="55"/>
+      <c r="S23" s="55"/>
+      <c r="T23" s="63"/>
+    </row>
+    <row r="24" spans="1:20" s="18" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="96"/>
+      <c r="B24" s="94"/>
+      <c r="C24" s="94"/>
+      <c r="D24" s="94"/>
+      <c r="E24" s="94"/>
+      <c r="F24" s="94"/>
+      <c r="G24" s="94"/>
+      <c r="H24" s="95" t="s">
+        <v>22</v>
+      </c>
+      <c r="I24" s="95"/>
+      <c r="J24" s="95"/>
+      <c r="K24" s="95"/>
+      <c r="L24" s="95"/>
+      <c r="M24" s="94"/>
+      <c r="N24" s="94"/>
+      <c r="O24" s="94"/>
+      <c r="P24" s="94"/>
+      <c r="Q24" s="69" t="s">
         <v>47</v>
       </c>
-      <c r="N20" s="95"/>
-      <c r="O20" s="95"/>
-      <c r="P20" s="96"/>
-      <c r="Q20" s="94" t="s">
-        <v>34</v>
-      </c>
-      <c r="R20" s="95"/>
-      <c r="S20" s="95"/>
-      <c r="T20" s="96"/>
-    </row>
-    <row r="21" spans="1:20" s="18" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="79"/>
-      <c r="B21" s="80"/>
-      <c r="C21" s="79"/>
-      <c r="D21" s="80"/>
-      <c r="E21" s="97"/>
-      <c r="F21" s="98"/>
-      <c r="G21" s="99"/>
-      <c r="H21" s="79"/>
-      <c r="I21" s="92"/>
-      <c r="J21" s="92"/>
-      <c r="K21" s="92"/>
-      <c r="L21" s="80"/>
-      <c r="M21" s="79"/>
-      <c r="N21" s="92"/>
-      <c r="O21" s="92"/>
-      <c r="P21" s="80"/>
-      <c r="Q21" s="79"/>
-      <c r="R21" s="92"/>
-      <c r="S21" s="92"/>
-      <c r="T21" s="80"/>
-    </row>
-    <row r="22" spans="1:20" s="18" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="46"/>
-      <c r="B22" s="7"/>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="42"/>
-      <c r="F22" s="42"/>
-      <c r="G22" s="42"/>
-      <c r="H22" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="I22" s="7"/>
-      <c r="J22" s="7"/>
-      <c r="K22" s="7"/>
-      <c r="L22" s="7"/>
-      <c r="M22" s="7"/>
-      <c r="N22" s="7"/>
-      <c r="O22" s="7"/>
-      <c r="P22" s="7"/>
-      <c r="Q22" s="49" t="s">
-        <v>37</v>
-      </c>
-      <c r="R22" s="49"/>
-      <c r="S22" s="49"/>
-      <c r="T22" s="50"/>
-    </row>
-    <row r="23" spans="1:20" s="18" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="47"/>
-      <c r="B23" s="7"/>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="42"/>
-      <c r="F23" s="42"/>
-      <c r="G23" s="42"/>
-      <c r="H23" s="31" t="s">
-        <v>36</v>
-      </c>
-      <c r="I23" s="7"/>
-      <c r="J23" s="7"/>
-      <c r="K23" s="7"/>
-      <c r="L23" s="7"/>
-      <c r="M23" s="7"/>
-      <c r="N23" s="7"/>
-      <c r="O23" s="7"/>
-      <c r="P23" s="7"/>
-      <c r="Q23" s="51" t="s">
-        <v>38</v>
-      </c>
-      <c r="R23" s="51"/>
-      <c r="S23" s="51"/>
-      <c r="T23" s="52"/>
-    </row>
-    <row r="24" spans="1:20" s="18" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A24" s="48"/>
-      <c r="B24" s="43"/>
-      <c r="C24" s="43"/>
-      <c r="D24" s="43"/>
-      <c r="E24" s="43"/>
-      <c r="F24" s="43"/>
-      <c r="G24" s="43"/>
-      <c r="H24" s="44" t="s">
-        <v>23</v>
-      </c>
-      <c r="I24" s="43"/>
-      <c r="J24" s="44" t="s">
-        <v>19</v>
-      </c>
-      <c r="K24" s="43"/>
-      <c r="L24" s="43"/>
-      <c r="M24" s="43"/>
-      <c r="N24" s="43"/>
-      <c r="O24" s="43"/>
-      <c r="P24" s="45"/>
-      <c r="Q24" s="56" t="s">
-        <v>48</v>
-      </c>
-      <c r="R24" s="56"/>
-      <c r="S24" s="56"/>
-      <c r="T24" s="57"/>
+      <c r="R24" s="69"/>
+      <c r="S24" s="69"/>
+      <c r="T24" s="70"/>
     </row>
     <row r="25" spans="1:20" s="18" customFormat="1" ht="18" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="5"/>
-      <c r="B25" s="5"/>
-      <c r="C25" s="5"/>
-      <c r="D25" s="5"/>
-      <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
-      <c r="G25" s="5"/>
-      <c r="I25" s="5"/>
-      <c r="K25" s="5"/>
-      <c r="L25" s="5"/>
-      <c r="M25" s="5"/>
-      <c r="N25" s="5"/>
-      <c r="O25" s="5"/>
-      <c r="P25" s="36"/>
-      <c r="Q25" s="37"/>
-      <c r="R25" s="37"/>
-      <c r="S25" s="37"/>
-      <c r="T25" s="37"/>
+      <c r="A25" s="100"/>
+      <c r="B25" s="100"/>
+      <c r="C25" s="100"/>
+      <c r="D25" s="100"/>
+      <c r="E25" s="100"/>
+      <c r="F25" s="100"/>
+      <c r="G25" s="100"/>
+      <c r="H25" s="99"/>
+      <c r="I25" s="99"/>
+      <c r="J25" s="99"/>
+      <c r="K25" s="99"/>
+      <c r="L25" s="99"/>
+      <c r="M25" s="100"/>
+      <c r="N25" s="100"/>
+      <c r="O25" s="100"/>
+      <c r="P25" s="100"/>
+      <c r="Q25" s="101"/>
+      <c r="R25" s="101"/>
+      <c r="S25" s="101"/>
+      <c r="T25" s="101"/>
     </row>
     <row r="26" spans="1:20" s="18" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="27" t="s">
@@ -2692,7 +2716,7 @@
         <v>8</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H26" s="10"/>
       <c r="I26" s="10"/>
@@ -2720,7 +2744,7 @@
         <v>8</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H27" s="5"/>
       <c r="I27" s="5"/>
@@ -2748,7 +2772,7 @@
         <v>8</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H28" s="5"/>
       <c r="I28" s="5"/>
@@ -2776,7 +2800,7 @@
         <v>8</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H29" s="8"/>
       <c r="I29" s="8"/>
@@ -2815,92 +2839,92 @@
       <c r="T30" s="5"/>
     </row>
     <row r="31" spans="1:20" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A31" s="39" t="s">
+      <c r="A31" s="37" t="s">
+        <v>29</v>
+      </c>
+      <c r="B31" s="37"/>
+      <c r="C31" s="37"/>
+      <c r="D31" s="37"/>
+      <c r="E31" s="37"/>
+      <c r="F31" s="37"/>
+      <c r="G31" s="37"/>
+      <c r="H31" s="37"/>
+      <c r="I31" s="37"/>
+      <c r="J31" s="37"/>
+    </row>
+    <row r="32" spans="1:20" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A32" s="37"/>
+      <c r="B32" s="37"/>
+      <c r="C32" s="37"/>
+      <c r="D32" s="37"/>
+      <c r="E32" s="37"/>
+      <c r="F32" s="37"/>
+      <c r="G32" s="37"/>
+      <c r="H32" s="37"/>
+      <c r="I32" s="37"/>
+      <c r="J32" s="37"/>
+    </row>
+    <row r="33" spans="1:20" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A33" s="38">
+        <v>1</v>
+      </c>
+      <c r="B33" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="B31" s="39"/>
-      <c r="C31" s="39"/>
-      <c r="D31" s="39"/>
-      <c r="E31" s="39"/>
-      <c r="F31" s="39"/>
-      <c r="G31" s="39"/>
-      <c r="H31" s="39"/>
-      <c r="I31" s="39"/>
-      <c r="J31" s="39"/>
-    </row>
-    <row r="32" spans="1:20" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A32" s="39"/>
-      <c r="B32" s="39"/>
-      <c r="C32" s="39"/>
-      <c r="D32" s="39"/>
-      <c r="E32" s="39"/>
-      <c r="F32" s="39"/>
-      <c r="G32" s="39"/>
-      <c r="H32" s="39"/>
-      <c r="I32" s="39"/>
-      <c r="J32" s="39"/>
-    </row>
-    <row r="33" spans="1:20" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A33" s="40">
-        <v>1</v>
-      </c>
-      <c r="B33" s="39" t="s">
+      <c r="C33" s="37"/>
+      <c r="D33" s="37"/>
+      <c r="E33" s="37"/>
+      <c r="F33" s="37"/>
+      <c r="G33" s="37"/>
+      <c r="H33" s="37"/>
+      <c r="I33" s="37"/>
+      <c r="J33" s="37"/>
+    </row>
+    <row r="34" spans="1:20" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A34" s="38">
+        <v>2</v>
+      </c>
+      <c r="B34" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="C33" s="39"/>
-      <c r="D33" s="39"/>
-      <c r="E33" s="39"/>
-      <c r="F33" s="39"/>
-      <c r="G33" s="39"/>
-      <c r="H33" s="39"/>
-      <c r="I33" s="39"/>
-      <c r="J33" s="39"/>
-    </row>
-    <row r="34" spans="1:20" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A34" s="40">
-        <v>2</v>
-      </c>
-      <c r="B34" s="39" t="s">
+      <c r="C34" s="37"/>
+      <c r="D34" s="37"/>
+      <c r="E34" s="37"/>
+      <c r="F34" s="37"/>
+      <c r="G34" s="37"/>
+      <c r="H34" s="37"/>
+      <c r="I34" s="37"/>
+      <c r="J34" s="37"/>
+    </row>
+    <row r="35" spans="1:20" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A35" s="38">
+        <v>3</v>
+      </c>
+      <c r="B35" s="37" t="s">
         <v>32</v>
       </c>
-      <c r="C34" s="39"/>
-      <c r="D34" s="39"/>
-      <c r="E34" s="39"/>
-      <c r="F34" s="39"/>
-      <c r="G34" s="39"/>
-      <c r="H34" s="39"/>
-      <c r="I34" s="39"/>
-      <c r="J34" s="39"/>
-    </row>
-    <row r="35" spans="1:20" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A35" s="40">
-        <v>3</v>
-      </c>
-      <c r="B35" s="39" t="s">
-        <v>33</v>
-      </c>
-      <c r="C35" s="39"/>
-      <c r="D35" s="39"/>
-      <c r="E35" s="39"/>
-      <c r="F35" s="39"/>
-      <c r="G35" s="39"/>
-      <c r="H35" s="39"/>
-      <c r="I35" s="39"/>
-      <c r="J35" s="39"/>
+      <c r="C35" s="37"/>
+      <c r="D35" s="37"/>
+      <c r="E35" s="37"/>
+      <c r="F35" s="37"/>
+      <c r="G35" s="37"/>
+      <c r="H35" s="37"/>
+      <c r="I35" s="37"/>
+      <c r="J35" s="37"/>
     </row>
     <row r="36" spans="1:20" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A36" s="39"/>
-      <c r="B36" s="39" t="s">
-        <v>29</v>
-      </c>
-      <c r="C36" s="39"/>
-      <c r="D36" s="39"/>
-      <c r="E36" s="39"/>
-      <c r="F36" s="39"/>
-      <c r="G36" s="39"/>
-      <c r="H36" s="39"/>
-      <c r="I36" s="39"/>
-      <c r="J36" s="39"/>
+      <c r="A36" s="37"/>
+      <c r="B36" s="37" t="s">
+        <v>28</v>
+      </c>
+      <c r="C36" s="37"/>
+      <c r="D36" s="37"/>
+      <c r="E36" s="37"/>
+      <c r="F36" s="37"/>
+      <c r="G36" s="37"/>
+      <c r="H36" s="37"/>
+      <c r="I36" s="37"/>
+      <c r="J36" s="37"/>
     </row>
     <row r="37" spans="1:20" s="18" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="5"/>
@@ -2948,7 +2972,7 @@
     </row>
     <row r="39" spans="1:20" s="18" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B39" s="5"/>
       <c r="C39" s="5"/>
@@ -2972,7 +2996,7 @@
     </row>
     <row r="40" spans="1:20" s="18" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B40" s="5"/>
       <c r="C40" s="5"/>
@@ -3017,8 +3041,8 @@
       <c r="T41" s="5"/>
     </row>
     <row r="42" spans="1:20" s="18" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="38" t="s">
-        <v>28</v>
+      <c r="A42" s="36" t="s">
+        <v>27</v>
       </c>
       <c r="B42" s="5"/>
       <c r="C42" s="5"/>
@@ -3063,14 +3087,14 @@
       <c r="T43" s="5"/>
     </row>
     <row r="44" spans="1:20" s="18" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="55" t="s">
-        <v>27</v>
-      </c>
-      <c r="B44" s="55"/>
-      <c r="C44" s="55"/>
-      <c r="D44" s="55"/>
-      <c r="E44" s="55"/>
-      <c r="F44" s="55"/>
+      <c r="A44" s="68" t="s">
+        <v>26</v>
+      </c>
+      <c r="B44" s="68"/>
+      <c r="C44" s="68"/>
+      <c r="D44" s="68"/>
+      <c r="E44" s="68"/>
+      <c r="F44" s="68"/>
       <c r="G44" s="5"/>
       <c r="H44" s="5"/>
       <c r="I44" s="5"/>
@@ -3088,7 +3112,7 @@
     </row>
     <row r="45" spans="1:20" s="18" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="31" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B45" s="31"/>
       <c r="C45" s="31"/>
@@ -3669,28 +3693,26 @@
       <c r="W76" s="33"/>
     </row>
   </sheetData>
-  <mergeCells count="35">
-    <mergeCell ref="E21:G21"/>
-    <mergeCell ref="H21:L21"/>
-    <mergeCell ref="Q19:T19"/>
-    <mergeCell ref="M19:P19"/>
-    <mergeCell ref="H19:L19"/>
-    <mergeCell ref="H20:L20"/>
-    <mergeCell ref="M20:P20"/>
-    <mergeCell ref="Q20:T20"/>
-    <mergeCell ref="M21:P21"/>
-    <mergeCell ref="Q21:T21"/>
-    <mergeCell ref="A3:T3"/>
-    <mergeCell ref="A4:T4"/>
-    <mergeCell ref="A5:T5"/>
-    <mergeCell ref="A6:T6"/>
-    <mergeCell ref="N12:S12"/>
-    <mergeCell ref="E19:G19"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="C20:D20"/>
+  <mergeCells count="56">
+    <mergeCell ref="H25:L25"/>
+    <mergeCell ref="M25:P25"/>
+    <mergeCell ref="Q25:T25"/>
+    <mergeCell ref="E25:G25"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="E22:G22"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="M23:P23"/>
+    <mergeCell ref="M24:P24"/>
+    <mergeCell ref="H23:L23"/>
+    <mergeCell ref="H24:L24"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="E23:G23"/>
+    <mergeCell ref="E24:G24"/>
     <mergeCell ref="Q22:T22"/>
     <mergeCell ref="Q23:T23"/>
     <mergeCell ref="K14:N14"/>
@@ -3705,6 +3727,29 @@
     <mergeCell ref="H17:L18"/>
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="E20:G20"/>
+    <mergeCell ref="M22:P22"/>
+    <mergeCell ref="H22:L22"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="A3:T3"/>
+    <mergeCell ref="A4:T4"/>
+    <mergeCell ref="A5:T5"/>
+    <mergeCell ref="A6:T6"/>
+    <mergeCell ref="N12:S12"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="H21:L21"/>
+    <mergeCell ref="Q19:T19"/>
+    <mergeCell ref="M19:P19"/>
+    <mergeCell ref="H19:L19"/>
+    <mergeCell ref="H20:L20"/>
+    <mergeCell ref="M20:P20"/>
+    <mergeCell ref="Q20:T20"/>
+    <mergeCell ref="M21:P21"/>
+    <mergeCell ref="Q21:T21"/>
+    <mergeCell ref="E19:G19"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>